<commit_message>
added more lcoe lc_summary
</commit_message>
<xml_diff>
--- a/lcoe_plots/bio_ethanol_lcoe/LCOE_BIOETHANOL.xlsx
+++ b/lcoe_plots/bio_ethanol_lcoe/LCOE_BIOETHANOL.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abbie/MacroEnergy-Abbie.jl/MacroEnergyExamples/lcoe_plots/bio_ethanol_lcoe/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95091DDC-D7CF-3845-89B4-AAB615614D65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97023F85-A260-3444-A124-FCACA1BD8636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29400" yWindow="500" windowWidth="38400" windowHeight="20460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Analysis" sheetId="2" r:id="rId2"/>
+    <sheet name="lc_detailed" sheetId="1" r:id="rId1"/>
+    <sheet name="lc_summary" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="80">
   <si>
     <t>Asset Parameters (normalized by commodity feedstock)</t>
   </si>
@@ -252,80 +252,6 @@
     <t>Biomass_Agri</t>
   </si>
   <si>
-    <t>Table 1 — Sorted by AM, AN</t>
-  </si>
-  <si>
-    <t>Table 2 — Sorted by AN</t>
-  </si>
-  <si>
-    <t>AK
-id_LC</t>
-  </si>
-  <si>
-    <t>AL
-commodity_LC</t>
-  </si>
-  <si>
-    <t>AR
-elec_production</t>
-  </si>
-  <si>
-    <t>AS
-elec_consumption</t>
-  </si>
-  <si>
-    <t>AT
-biomass_consumption</t>
-  </si>
-  <si>
-    <t>AU
-natgas_consumption</t>
-  </si>
-  <si>
-    <t>AV
-investment_cost</t>
-  </si>
-  <si>
-    <t>AW
-fixed_om_cost</t>
-  </si>
-  <si>
-    <t>AX
-variable_om_cost</t>
-  </si>
-  <si>
-    <t>AY
-CI</t>
-  </si>
-  <si>
-    <t>AZ
-modified capture cost</t>
-  </si>
-  <si>
-    <t>BA
-modified emissions cost</t>
-  </si>
-  <si>
-    <t>AM
-LCOE ($/MWh-ethanol)</t>
-  </si>
-  <si>
-    <t>AN
-LCOE ($/MWh-ethanol)</t>
-  </si>
-  <si>
-    <t>BB
-CI</t>
-  </si>
-  <si>
-    <t>BC
-modified capture cost</t>
-  </si>
-  <si>
-    <t>BD
-modified emissions cost</t>
-  </si>
-  <si>
     <t>calculated_emission_rate (t-CO2/t-bio)</t>
   </si>
   <si>
@@ -336,6 +262,18 @@
   </si>
   <si>
     <t>Total input (t-CO2/MWh-ethanol)</t>
+  </si>
+  <si>
+    <t>LC for bioethanol production $/GJ</t>
+  </si>
+  <si>
+    <t>CHECK LCOE ($/GJ-ethanol)</t>
+  </si>
+  <si>
+    <t>Conversion</t>
+  </si>
+  <si>
+    <t>GJ/MWh</t>
   </si>
 </sst>
 </file>
@@ -345,7 +283,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -383,19 +321,14 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <name val="Arial"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -476,17 +409,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E79"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFF7E9FF"/>
         <bgColor rgb="FFADD8E6"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -494,26 +422,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB0C4D8"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB0C4D8"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB0C4D8"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB0C4D8"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -532,14 +445,13 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -984,7 +896,7 @@
         <v>9</v>
       </c>
       <c r="BT2" s="1" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="2:72" x14ac:dyDescent="0.2">
@@ -1016,7 +928,7 @@
         <v>18</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>19</v>
@@ -1166,7 +1078,7 @@
         <v>61</v>
       </c>
       <c r="BM3" s="7" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="BO3" s="7" t="s">
         <v>59</v>
@@ -1181,7 +1093,7 @@
         <v>64</v>
       </c>
       <c r="BT3" s="7" t="s">
-        <v>93</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="2:72" x14ac:dyDescent="0.2">
@@ -1213,7 +1125,7 @@
         <f>K4</f>
         <v>1.0345289563701205</v>
       </c>
-      <c r="K4" s="21">
+      <c r="K4" s="18">
         <f>(BL4+(BK4-BO4-BQ4))*F4</f>
         <v>1.0345289563701205</v>
       </c>
@@ -1274,11 +1186,11 @@
         <v>576.81126900000004</v>
       </c>
       <c r="AL4" s="1" t="str">
-        <f>B4</f>
+        <f t="shared" ref="AL4:AM7" si="0">B4</f>
         <v>SE_DryMill_Existing_Non_CCS</v>
       </c>
       <c r="AM4" s="1" t="str">
-        <f>C4</f>
+        <f t="shared" si="0"/>
         <v>Biomass_Corn</v>
       </c>
       <c r="AN4" s="11">
@@ -1290,11 +1202,11 @@
         <v>37.095845147977556</v>
       </c>
       <c r="AP4" s="11">
-        <f t="shared" ref="AP4:AQ7" si="0">AN4/3.6</f>
+        <f t="shared" ref="AP4:AQ7" si="1">AN4/3.6</f>
         <v>10.304401429993765</v>
       </c>
       <c r="AQ4" s="11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>10.304401429993765</v>
       </c>
       <c r="AR4" s="5">
@@ -1422,11 +1334,11 @@
         <v>0</v>
       </c>
       <c r="J5" s="12">
-        <f t="shared" ref="J5:J7" si="1">K5</f>
+        <f t="shared" ref="J5:J7" si="2">K5</f>
         <v>0.9625997476999999</v>
       </c>
-      <c r="K5" s="21">
-        <f t="shared" ref="K5:K7" si="2">(BL5+(BK5-BO5-BQ5))*F5</f>
+      <c r="K5" s="18">
+        <f t="shared" ref="K5:K7" si="3">(BL5+(BK5-BO5-BQ5))*F5</f>
         <v>0.9625997476999999</v>
       </c>
       <c r="L5" s="12">
@@ -1486,11 +1398,11 @@
         <v>576.81126900000004</v>
       </c>
       <c r="AL5" s="1" t="str">
-        <f>B5</f>
+        <f t="shared" si="0"/>
         <v>SE_Biochemical_Non_CCS</v>
       </c>
       <c r="AM5" s="1" t="str">
-        <f>C5</f>
+        <f t="shared" si="0"/>
         <v>Biomass_Herb</v>
       </c>
       <c r="AN5" s="11">
@@ -1502,11 +1414,11 @@
         <v>150.7032182807072</v>
       </c>
       <c r="AP5" s="11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>41.862005077974224</v>
       </c>
       <c r="AQ5" s="11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>41.862005077974224</v>
       </c>
       <c r="AR5" s="5">
@@ -1604,7 +1516,7 @@
         <v>0.851118705267909</v>
       </c>
       <c r="BT5" s="1">
-        <f t="shared" ref="BT5:BT7" si="3">BM5-BR5</f>
+        <f t="shared" ref="BT5:BT7" si="4">BM5-BR5</f>
         <v>0</v>
       </c>
     </row>
@@ -1634,11 +1546,11 @@
         <v>0.19</v>
       </c>
       <c r="J6" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.77259974769999995</v>
       </c>
-      <c r="K6" s="21">
-        <f t="shared" si="2"/>
+      <c r="K6" s="18">
+        <f t="shared" si="3"/>
         <v>0.77259974769999995</v>
       </c>
       <c r="L6" s="12">
@@ -1698,11 +1610,11 @@
         <v>576.81126900000004</v>
       </c>
       <c r="AL6" s="1" t="str">
-        <f>B6</f>
+        <f t="shared" si="0"/>
         <v>SE_Biochemical_CCS_20</v>
       </c>
       <c r="AM6" s="1" t="str">
-        <f>C6</f>
+        <f t="shared" si="0"/>
         <v>Biomass_Herb</v>
       </c>
       <c r="AN6" s="11">
@@ -1714,11 +1626,11 @@
         <v>137.19357300111162</v>
       </c>
       <c r="AP6" s="11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>38.109325833642117</v>
       </c>
       <c r="AQ6" s="11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>38.109325833642117</v>
       </c>
       <c r="AR6" s="5">
@@ -1816,7 +1728,7 @@
         <v>0.851118705267909</v>
       </c>
       <c r="BT6" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -1846,11 +1758,11 @@
         <v>0.83</v>
       </c>
       <c r="J7" s="12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.13259974769999996</v>
       </c>
-      <c r="K7" s="21">
-        <f t="shared" si="2"/>
+      <c r="K7" s="18">
+        <f t="shared" si="3"/>
         <v>0.13259974769999996</v>
       </c>
       <c r="L7" s="12">
@@ -1910,11 +1822,11 @@
         <v>576.81126900000004</v>
       </c>
       <c r="AL7" s="1" t="str">
-        <f>B7</f>
+        <f t="shared" si="0"/>
         <v>SE_Biochemical_CCS_86</v>
       </c>
       <c r="AM7" s="1" t="str">
-        <f>C7</f>
+        <f t="shared" si="0"/>
         <v>Biomass_Agri</v>
       </c>
       <c r="AN7" s="11">
@@ -1926,11 +1838,11 @@
         <v>96.119178840263785</v>
       </c>
       <c r="AP7" s="11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>26.699771900073276</v>
       </c>
       <c r="AQ7" s="11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>26.699771900073273</v>
       </c>
       <c r="AR7" s="5">
@@ -2028,7 +1940,7 @@
         <v>0.851118705267909</v>
       </c>
       <c r="BT7" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -2042,7 +1954,7 @@
       <c r="H8" s="12"/>
       <c r="I8" s="12"/>
       <c r="J8" s="12"/>
-      <c r="K8" s="21"/>
+      <c r="K8" s="18"/>
       <c r="L8" s="12"/>
       <c r="M8" s="12"/>
       <c r="N8" s="12"/>
@@ -2093,7 +2005,7 @@
       <c r="H9" s="12"/>
       <c r="I9" s="12"/>
       <c r="J9" s="12"/>
-      <c r="K9" s="21"/>
+      <c r="K9" s="18"/>
       <c r="L9" s="12"/>
       <c r="M9" s="12"/>
       <c r="N9" s="12"/>
@@ -2144,7 +2056,7 @@
       <c r="H10" s="12"/>
       <c r="I10" s="12"/>
       <c r="J10" s="12"/>
-      <c r="K10" s="21"/>
+      <c r="K10" s="18"/>
       <c r="L10" s="12"/>
       <c r="M10" s="12"/>
       <c r="N10" s="12"/>
@@ -2195,7 +2107,7 @@
       <c r="H11" s="12"/>
       <c r="I11" s="12"/>
       <c r="J11" s="12"/>
-      <c r="K11" s="21"/>
+      <c r="K11" s="18"/>
       <c r="L11" s="12"/>
       <c r="M11" s="12"/>
       <c r="N11" s="12"/>
@@ -2246,7 +2158,7 @@
       <c r="H12" s="12"/>
       <c r="I12" s="12"/>
       <c r="J12" s="12"/>
-      <c r="K12" s="21"/>
+      <c r="K12" s="18"/>
       <c r="L12" s="12"/>
       <c r="M12" s="12"/>
       <c r="N12" s="12"/>
@@ -2297,7 +2209,7 @@
       <c r="H13" s="12"/>
       <c r="I13" s="12"/>
       <c r="J13" s="12"/>
-      <c r="K13" s="21"/>
+      <c r="K13" s="18"/>
       <c r="L13" s="12"/>
       <c r="M13" s="12"/>
       <c r="N13" s="12"/>
@@ -2348,7 +2260,7 @@
       <c r="H14" s="12"/>
       <c r="I14" s="12"/>
       <c r="J14" s="12"/>
-      <c r="K14" s="21"/>
+      <c r="K14" s="18"/>
       <c r="L14" s="12"/>
       <c r="M14" s="12"/>
       <c r="N14" s="12"/>
@@ -2399,7 +2311,7 @@
       <c r="H15" s="12"/>
       <c r="I15" s="12"/>
       <c r="J15" s="12"/>
-      <c r="K15" s="21"/>
+      <c r="K15" s="18"/>
       <c r="L15" s="12"/>
       <c r="M15" s="12"/>
       <c r="N15" s="12"/>
@@ -2450,7 +2362,7 @@
       <c r="H16" s="12"/>
       <c r="I16" s="12"/>
       <c r="J16" s="12"/>
-      <c r="K16" s="21"/>
+      <c r="K16" s="18"/>
       <c r="L16" s="12"/>
       <c r="M16" s="12"/>
       <c r="N16" s="12"/>
@@ -2501,7 +2413,7 @@
       <c r="H17" s="12"/>
       <c r="I17" s="12"/>
       <c r="J17" s="12"/>
-      <c r="K17" s="21"/>
+      <c r="K17" s="18"/>
       <c r="L17" s="12"/>
       <c r="M17" s="12"/>
       <c r="N17" s="12"/>
@@ -2552,7 +2464,7 @@
       <c r="H18" s="12"/>
       <c r="I18" s="12"/>
       <c r="J18" s="12"/>
-      <c r="K18" s="21"/>
+      <c r="K18" s="18"/>
       <c r="L18" s="12"/>
       <c r="M18" s="12"/>
       <c r="N18" s="12"/>
@@ -2603,7 +2515,7 @@
       <c r="H19" s="12"/>
       <c r="I19" s="12"/>
       <c r="J19" s="12"/>
-      <c r="K19" s="21"/>
+      <c r="K19" s="18"/>
       <c r="L19" s="12"/>
       <c r="M19" s="12"/>
       <c r="N19" s="12"/>
@@ -2654,7 +2566,7 @@
       <c r="H20" s="12"/>
       <c r="I20" s="12"/>
       <c r="J20" s="12"/>
-      <c r="K20" s="21"/>
+      <c r="K20" s="18"/>
       <c r="L20" s="12"/>
       <c r="M20" s="12"/>
       <c r="N20" s="12"/>
@@ -2705,7 +2617,7 @@
       <c r="H21" s="12"/>
       <c r="I21" s="12"/>
       <c r="J21" s="12"/>
-      <c r="K21" s="21"/>
+      <c r="K21" s="18"/>
       <c r="L21" s="12"/>
       <c r="M21" s="12"/>
       <c r="N21" s="12"/>
@@ -2756,7 +2668,7 @@
       <c r="H22" s="12"/>
       <c r="I22" s="12"/>
       <c r="J22" s="12"/>
-      <c r="K22" s="21"/>
+      <c r="K22" s="18"/>
       <c r="L22" s="12"/>
       <c r="M22" s="12"/>
       <c r="N22" s="12"/>
@@ -2807,7 +2719,7 @@
       <c r="H23" s="12"/>
       <c r="I23" s="12"/>
       <c r="J23" s="12"/>
-      <c r="K23" s="21"/>
+      <c r="K23" s="18"/>
       <c r="L23" s="12"/>
       <c r="M23" s="12"/>
       <c r="N23" s="12"/>
@@ -2858,7 +2770,7 @@
       <c r="H24" s="12"/>
       <c r="I24" s="12"/>
       <c r="J24" s="12"/>
-      <c r="K24" s="21"/>
+      <c r="K24" s="18"/>
       <c r="L24" s="12"/>
       <c r="M24" s="12"/>
       <c r="N24" s="12"/>
@@ -2909,7 +2821,7 @@
       <c r="H25" s="12"/>
       <c r="I25" s="12"/>
       <c r="J25" s="12"/>
-      <c r="K25" s="21"/>
+      <c r="K25" s="18"/>
       <c r="L25" s="12"/>
       <c r="M25" s="12"/>
       <c r="N25" s="12"/>
@@ -2960,7 +2872,7 @@
       <c r="H26" s="12"/>
       <c r="I26" s="12"/>
       <c r="J26" s="12"/>
-      <c r="K26" s="21"/>
+      <c r="K26" s="18"/>
       <c r="L26" s="12"/>
       <c r="M26" s="12"/>
       <c r="N26" s="12"/>
@@ -3011,7 +2923,7 @@
       <c r="H27" s="12"/>
       <c r="I27" s="12"/>
       <c r="J27" s="12"/>
-      <c r="K27" s="21"/>
+      <c r="K27" s="18"/>
       <c r="L27" s="12"/>
       <c r="M27" s="12"/>
       <c r="N27" s="12"/>
@@ -3062,7 +2974,7 @@
       <c r="H28" s="12"/>
       <c r="I28" s="12"/>
       <c r="J28" s="12"/>
-      <c r="K28" s="21"/>
+      <c r="K28" s="18"/>
       <c r="L28" s="12"/>
       <c r="M28" s="12"/>
       <c r="N28" s="12"/>
@@ -3113,7 +3025,7 @@
       <c r="H29" s="12"/>
       <c r="I29" s="12"/>
       <c r="J29" s="12"/>
-      <c r="K29" s="21"/>
+      <c r="K29" s="18"/>
       <c r="L29" s="12"/>
       <c r="M29" s="12"/>
       <c r="N29" s="12"/>
@@ -3164,7 +3076,7 @@
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
       <c r="J30" s="12"/>
-      <c r="K30" s="21"/>
+      <c r="K30" s="18"/>
       <c r="L30" s="12"/>
       <c r="M30" s="12"/>
       <c r="N30" s="12"/>
@@ -3215,7 +3127,7 @@
       <c r="H31" s="12"/>
       <c r="I31" s="12"/>
       <c r="J31" s="12"/>
-      <c r="K31" s="21"/>
+      <c r="K31" s="18"/>
       <c r="L31" s="12"/>
       <c r="M31" s="12"/>
       <c r="N31" s="12"/>
@@ -3266,7 +3178,7 @@
       <c r="H32" s="12"/>
       <c r="I32" s="12"/>
       <c r="J32" s="12"/>
-      <c r="K32" s="21"/>
+      <c r="K32" s="18"/>
       <c r="L32" s="12"/>
       <c r="M32" s="12"/>
       <c r="N32" s="12"/>
@@ -3317,7 +3229,7 @@
       <c r="H33" s="12"/>
       <c r="I33" s="12"/>
       <c r="J33" s="12"/>
-      <c r="K33" s="21"/>
+      <c r="K33" s="18"/>
       <c r="L33" s="12"/>
       <c r="M33" s="12"/>
       <c r="N33" s="12"/>
@@ -3368,7 +3280,7 @@
       <c r="H34" s="12"/>
       <c r="I34" s="12"/>
       <c r="J34" s="12"/>
-      <c r="K34" s="21"/>
+      <c r="K34" s="18"/>
       <c r="L34" s="12"/>
       <c r="M34" s="12"/>
       <c r="N34" s="12"/>
@@ -3419,7 +3331,7 @@
       <c r="H35" s="12"/>
       <c r="I35" s="12"/>
       <c r="J35" s="12"/>
-      <c r="K35" s="21"/>
+      <c r="K35" s="18"/>
       <c r="L35" s="12"/>
       <c r="M35" s="12"/>
       <c r="N35" s="12"/>
@@ -3470,7 +3382,7 @@
       <c r="H36" s="12"/>
       <c r="I36" s="12"/>
       <c r="J36" s="12"/>
-      <c r="K36" s="21"/>
+      <c r="K36" s="18"/>
       <c r="L36" s="12"/>
       <c r="M36" s="12"/>
       <c r="N36" s="12"/>
@@ -3521,7 +3433,7 @@
       <c r="H37" s="12"/>
       <c r="I37" s="12"/>
       <c r="J37" s="12"/>
-      <c r="K37" s="21"/>
+      <c r="K37" s="18"/>
       <c r="L37" s="12"/>
       <c r="M37" s="12"/>
       <c r="N37" s="12"/>
@@ -3572,7 +3484,7 @@
       <c r="H38" s="12"/>
       <c r="I38" s="12"/>
       <c r="J38" s="12"/>
-      <c r="K38" s="21"/>
+      <c r="K38" s="18"/>
       <c r="L38" s="12"/>
       <c r="M38" s="12"/>
       <c r="N38" s="12"/>
@@ -3623,7 +3535,7 @@
       <c r="H39" s="12"/>
       <c r="I39" s="12"/>
       <c r="J39" s="12"/>
-      <c r="K39" s="21"/>
+      <c r="K39" s="18"/>
       <c r="L39" s="12"/>
       <c r="M39" s="12"/>
       <c r="N39" s="12"/>
@@ -3674,7 +3586,7 @@
       <c r="H40" s="12"/>
       <c r="I40" s="12"/>
       <c r="J40" s="12"/>
-      <c r="K40" s="21"/>
+      <c r="K40" s="18"/>
       <c r="L40" s="12"/>
       <c r="M40" s="12"/>
       <c r="N40" s="12"/>
@@ -3725,7 +3637,7 @@
       <c r="H41" s="12"/>
       <c r="I41" s="12"/>
       <c r="J41" s="12"/>
-      <c r="K41" s="21"/>
+      <c r="K41" s="18"/>
       <c r="L41" s="12"/>
       <c r="M41" s="12"/>
       <c r="N41" s="12"/>
@@ -3776,7 +3688,7 @@
       <c r="H42" s="12"/>
       <c r="I42" s="12"/>
       <c r="J42" s="12"/>
-      <c r="K42" s="21"/>
+      <c r="K42" s="18"/>
       <c r="L42" s="12"/>
       <c r="M42" s="12"/>
       <c r="N42" s="12"/>
@@ -3827,7 +3739,7 @@
       <c r="H43" s="12"/>
       <c r="I43" s="12"/>
       <c r="J43" s="12"/>
-      <c r="K43" s="21"/>
+      <c r="K43" s="18"/>
       <c r="L43" s="12"/>
       <c r="M43" s="12"/>
       <c r="N43" s="12"/>
@@ -3878,7 +3790,7 @@
       <c r="H44" s="12"/>
       <c r="I44" s="12"/>
       <c r="J44" s="12"/>
-      <c r="K44" s="21"/>
+      <c r="K44" s="18"/>
       <c r="L44" s="12"/>
       <c r="M44" s="12"/>
       <c r="N44" s="12"/>
@@ -3929,7 +3841,7 @@
       <c r="H45" s="12"/>
       <c r="I45" s="12"/>
       <c r="J45" s="12"/>
-      <c r="K45" s="21"/>
+      <c r="K45" s="18"/>
       <c r="L45" s="12"/>
       <c r="M45" s="12"/>
       <c r="N45" s="12"/>
@@ -3980,7 +3892,7 @@
       <c r="H46" s="12"/>
       <c r="I46" s="12"/>
       <c r="J46" s="12"/>
-      <c r="K46" s="21"/>
+      <c r="K46" s="18"/>
       <c r="L46" s="12"/>
       <c r="M46" s="12"/>
       <c r="N46" s="12"/>
@@ -4031,7 +3943,7 @@
       <c r="H47" s="12"/>
       <c r="I47" s="12"/>
       <c r="J47" s="12"/>
-      <c r="K47" s="21"/>
+      <c r="K47" s="18"/>
       <c r="L47" s="12"/>
       <c r="M47" s="12"/>
       <c r="N47" s="12"/>
@@ -4082,7 +3994,7 @@
       <c r="H48" s="12"/>
       <c r="I48" s="12"/>
       <c r="J48" s="12"/>
-      <c r="K48" s="21"/>
+      <c r="K48" s="18"/>
       <c r="L48" s="12"/>
       <c r="M48" s="12"/>
       <c r="N48" s="12"/>
@@ -4133,7 +4045,7 @@
       <c r="H49" s="12"/>
       <c r="I49" s="12"/>
       <c r="J49" s="12"/>
-      <c r="K49" s="21"/>
+      <c r="K49" s="18"/>
       <c r="L49" s="12"/>
       <c r="M49" s="12"/>
       <c r="N49" s="12"/>
@@ -4184,7 +4096,7 @@
       <c r="H50" s="12"/>
       <c r="I50" s="12"/>
       <c r="J50" s="12"/>
-      <c r="K50" s="21"/>
+      <c r="K50" s="18"/>
       <c r="L50" s="12"/>
       <c r="M50" s="12"/>
       <c r="N50" s="12"/>
@@ -4235,7 +4147,7 @@
       <c r="H51" s="12"/>
       <c r="I51" s="12"/>
       <c r="J51" s="12"/>
-      <c r="K51" s="21"/>
+      <c r="K51" s="18"/>
       <c r="L51" s="12"/>
       <c r="M51" s="12"/>
       <c r="N51" s="12"/>
@@ -4286,7 +4198,7 @@
       <c r="H52" s="12"/>
       <c r="I52" s="12"/>
       <c r="J52" s="12"/>
-      <c r="K52" s="21"/>
+      <c r="K52" s="18"/>
       <c r="L52" s="12"/>
       <c r="M52" s="12"/>
       <c r="N52" s="12"/>
@@ -4337,7 +4249,7 @@
       <c r="H53" s="12"/>
       <c r="I53" s="12"/>
       <c r="J53" s="12"/>
-      <c r="K53" s="21"/>
+      <c r="K53" s="18"/>
       <c r="L53" s="12"/>
       <c r="M53" s="12"/>
       <c r="N53" s="12"/>
@@ -4388,7 +4300,7 @@
       <c r="H54" s="12"/>
       <c r="I54" s="12"/>
       <c r="J54" s="12"/>
-      <c r="K54" s="21"/>
+      <c r="K54" s="18"/>
       <c r="L54" s="12"/>
       <c r="M54" s="12"/>
       <c r="N54" s="12"/>
@@ -4439,7 +4351,7 @@
       <c r="H55" s="12"/>
       <c r="I55" s="12"/>
       <c r="J55" s="12"/>
-      <c r="K55" s="21"/>
+      <c r="K55" s="18"/>
       <c r="L55" s="12"/>
       <c r="M55" s="12"/>
       <c r="N55" s="12"/>
@@ -4490,7 +4402,7 @@
       <c r="H56" s="12"/>
       <c r="I56" s="12"/>
       <c r="J56" s="12"/>
-      <c r="K56" s="21"/>
+      <c r="K56" s="18"/>
       <c r="L56" s="12"/>
       <c r="M56" s="12"/>
       <c r="N56" s="12"/>
@@ -4541,7 +4453,7 @@
       <c r="H57" s="12"/>
       <c r="I57" s="12"/>
       <c r="J57" s="12"/>
-      <c r="K57" s="21"/>
+      <c r="K57" s="18"/>
       <c r="L57" s="12"/>
       <c r="M57" s="12"/>
       <c r="N57" s="12"/>
@@ -4592,7 +4504,7 @@
       <c r="H58" s="12"/>
       <c r="I58" s="12"/>
       <c r="J58" s="12"/>
-      <c r="K58" s="21"/>
+      <c r="K58" s="18"/>
       <c r="L58" s="12"/>
       <c r="M58" s="12"/>
       <c r="N58" s="12"/>
@@ -4643,7 +4555,7 @@
       <c r="H59" s="12"/>
       <c r="I59" s="12"/>
       <c r="J59" s="12"/>
-      <c r="K59" s="21"/>
+      <c r="K59" s="18"/>
       <c r="L59" s="12"/>
       <c r="M59" s="12"/>
       <c r="N59" s="12"/>
@@ -4694,7 +4606,7 @@
       <c r="H60" s="12"/>
       <c r="I60" s="12"/>
       <c r="J60" s="12"/>
-      <c r="K60" s="21"/>
+      <c r="K60" s="18"/>
       <c r="L60" s="12"/>
       <c r="M60" s="12"/>
       <c r="N60" s="12"/>
@@ -4745,7 +4657,7 @@
       <c r="H61" s="12"/>
       <c r="I61" s="12"/>
       <c r="J61" s="12"/>
-      <c r="K61" s="21"/>
+      <c r="K61" s="18"/>
       <c r="L61" s="12"/>
       <c r="M61" s="12"/>
       <c r="N61" s="12"/>
@@ -4796,7 +4708,7 @@
       <c r="H62" s="12"/>
       <c r="I62" s="12"/>
       <c r="J62" s="12"/>
-      <c r="K62" s="21"/>
+      <c r="K62" s="18"/>
       <c r="L62" s="12"/>
       <c r="M62" s="12"/>
       <c r="N62" s="12"/>
@@ -4847,7 +4759,7 @@
       <c r="H63" s="12"/>
       <c r="I63" s="12"/>
       <c r="J63" s="12"/>
-      <c r="K63" s="21"/>
+      <c r="K63" s="18"/>
       <c r="L63" s="12"/>
       <c r="M63" s="12"/>
       <c r="N63" s="12"/>
@@ -4898,7 +4810,7 @@
       <c r="H64" s="12"/>
       <c r="I64" s="12"/>
       <c r="J64" s="12"/>
-      <c r="K64" s="21"/>
+      <c r="K64" s="18"/>
       <c r="L64" s="12"/>
       <c r="M64" s="12"/>
       <c r="N64" s="12"/>
@@ -4949,7 +4861,7 @@
       <c r="H65" s="12"/>
       <c r="I65" s="12"/>
       <c r="J65" s="12"/>
-      <c r="K65" s="21"/>
+      <c r="K65" s="18"/>
       <c r="L65" s="12"/>
       <c r="M65" s="12"/>
       <c r="N65" s="12"/>
@@ -5000,7 +4912,7 @@
       <c r="H66" s="12"/>
       <c r="I66" s="12"/>
       <c r="J66" s="12"/>
-      <c r="K66" s="21"/>
+      <c r="K66" s="18"/>
       <c r="L66" s="12"/>
       <c r="M66" s="12"/>
       <c r="N66" s="12"/>
@@ -5410,137 +5322,346 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A2:AB3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC586433-3FF4-3B40-A873-F79B41C708D7}">
+  <dimension ref="B2:U7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="18" customWidth="1"/>
-    <col min="3" max="14" width="14" customWidth="1"/>
-    <col min="16" max="17" width="18" customWidth="1"/>
-    <col min="18" max="28" width="14" customWidth="1"/>
+    <col min="1" max="1" width="2.5" customWidth="1"/>
+    <col min="2" max="2" width="29" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.1640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="2.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A2" s="19" t="s">
-        <v>72</v>
-      </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
-      <c r="N2" s="20"/>
-      <c r="P2" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q2" s="20"/>
-      <c r="R2" s="20"/>
-      <c r="S2" s="20"/>
-      <c r="T2" s="20"/>
-      <c r="U2" s="20"/>
-      <c r="V2" s="20"/>
-      <c r="W2" s="20"/>
-      <c r="X2" s="20"/>
-      <c r="Y2" s="20"/>
-      <c r="Z2" s="20"/>
-      <c r="AA2" s="20"/>
-      <c r="AB2" s="20"/>
-    </row>
-    <row r="3" spans="1:28" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="18" t="s">
-        <v>74</v>
-      </c>
-      <c r="B3" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="C3" s="18" t="s">
+    <row r="2" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B2" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="R2" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="S2" s="22"/>
+      <c r="T2" s="22"/>
+      <c r="U2" s="22"/>
+    </row>
+    <row r="3" spans="2:21" ht="32" x14ac:dyDescent="0.2">
+      <c r="B3" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="N3" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="O3" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="P3" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="R3" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="S3" s="22">
+        <v>3.6</v>
+      </c>
+      <c r="T3" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="G3" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="H3" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="I3" s="18" t="s">
-        <v>82</v>
-      </c>
-      <c r="J3" s="18" t="s">
-        <v>83</v>
-      </c>
-      <c r="K3" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="L3" s="18" t="s">
-        <v>85</v>
-      </c>
-      <c r="M3" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="N3" s="18" t="s">
-        <v>87</v>
-      </c>
-      <c r="P3" s="18" t="s">
-        <v>74</v>
-      </c>
-      <c r="Q3" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="R3" s="18" t="s">
-        <v>76</v>
-      </c>
-      <c r="S3" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="T3" s="18" t="s">
-        <v>78</v>
-      </c>
-      <c r="U3" s="18" t="s">
-        <v>79</v>
-      </c>
-      <c r="V3" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="W3" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="X3" s="18" t="s">
-        <v>82</v>
-      </c>
-      <c r="Y3" s="18" t="s">
-        <v>88</v>
-      </c>
-      <c r="Z3" s="18" t="s">
-        <v>89</v>
-      </c>
-      <c r="AA3" s="18" t="s">
-        <v>90</v>
-      </c>
-      <c r="AB3" s="18" t="s">
-        <v>87</v>
+      <c r="U3" s="22"/>
+    </row>
+    <row r="4" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B4" s="21" t="str">
+        <f>lc_detailed!AL4</f>
+        <v>SE_DryMill_Existing_Non_CCS</v>
+      </c>
+      <c r="C4" s="21" t="str">
+        <f>lc_detailed!AM4</f>
+        <v>Biomass_Corn</v>
+      </c>
+      <c r="D4" s="21">
+        <f>lc_detailed!AS4/$S$3</f>
+        <v>0</v>
+      </c>
+      <c r="E4" s="21">
+        <f>lc_detailed!AT4/$S$3</f>
+        <v>0.13576824642126792</v>
+      </c>
+      <c r="F4" s="21">
+        <f>lc_detailed!AU4/$S$3</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="21">
+        <f>lc_detailed!AV4/$S$3</f>
+        <v>0.30385250511247447</v>
+      </c>
+      <c r="H4" s="21">
+        <f>lc_detailed!AW4/$S$3</f>
+        <v>0</v>
+      </c>
+      <c r="I4" s="21">
+        <f>lc_detailed!AX4/$S$3</f>
+        <v>1.6648573495991814</v>
+      </c>
+      <c r="J4" s="21">
+        <f>lc_detailed!AY4/$S$3</f>
+        <v>6.7868098159509209</v>
+      </c>
+      <c r="K4" s="21">
+        <f>lc_detailed!BA4/$S$3</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="21">
+        <f>lc_detailed!BB4/$S$3</f>
+        <v>1.4131135129099206</v>
+      </c>
+      <c r="M4" s="21">
+        <f>lc_detailed!AZ4</f>
+        <v>4.1652201340527828E-2</v>
+      </c>
+      <c r="N4" s="21">
+        <f>lc_detailed!AN4</f>
+        <v>37.095845147977556</v>
+      </c>
+      <c r="O4" s="21">
+        <f>N4/$S$3</f>
+        <v>10.304401429993765</v>
+      </c>
+      <c r="P4" s="21">
+        <f>SUM(D4:L4)</f>
+        <v>10.304401429993764</v>
+      </c>
+    </row>
+    <row r="5" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B5" s="21" t="str">
+        <f>lc_detailed!AL5</f>
+        <v>SE_Biochemical_Non_CCS</v>
+      </c>
+      <c r="C5" s="21" t="str">
+        <f>lc_detailed!AM5</f>
+        <v>Biomass_Herb</v>
+      </c>
+      <c r="D5" s="21">
+        <f>lc_detailed!AS5/$S$3</f>
+        <v>-0.58361349436886112</v>
+      </c>
+      <c r="E5" s="21">
+        <f>lc_detailed!AT5/$S$3</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="21">
+        <f>lc_detailed!AU5/$S$3</f>
+        <v>13.128134918076242</v>
+      </c>
+      <c r="G5" s="21">
+        <f>lc_detailed!AV5/$S$3</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="21">
+        <f>lc_detailed!AW5/$S$3</f>
+        <v>14.915087692090401</v>
+      </c>
+      <c r="I5" s="21">
+        <f>lc_detailed!AX5/$S$3</f>
+        <v>4.4296919408554887</v>
+      </c>
+      <c r="J5" s="21">
+        <f>lc_detailed!AY5/$S$3</f>
+        <v>9.9727040213209541</v>
+      </c>
+      <c r="K5" s="21">
+        <f>lc_detailed!BA5/$S$3</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="21">
+        <f>lc_detailed!BB5/$S$3</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="21">
+        <f>lc_detailed!AZ5</f>
+        <v>0</v>
+      </c>
+      <c r="N5" s="21">
+        <f>lc_detailed!AN5</f>
+        <v>150.7032182807072</v>
+      </c>
+      <c r="O5" s="21">
+        <f t="shared" ref="O5:O37" si="0">N5/$S$3</f>
+        <v>41.862005077974224</v>
+      </c>
+      <c r="P5" s="21">
+        <f t="shared" ref="P5:P37" si="1">SUM(D5:L5)</f>
+        <v>41.862005077974224</v>
+      </c>
+    </row>
+    <row r="6" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B6" s="21" t="str">
+        <f>lc_detailed!AL6</f>
+        <v>SE_Biochemical_CCS_20</v>
+      </c>
+      <c r="C6" s="21" t="str">
+        <f>lc_detailed!AM6</f>
+        <v>Biomass_Herb</v>
+      </c>
+      <c r="D6" s="21">
+        <f>lc_detailed!AS6/$S$3</f>
+        <v>-0.58361349436886112</v>
+      </c>
+      <c r="E6" s="21">
+        <f>lc_detailed!AT6/$S$3</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="21">
+        <f>lc_detailed!AU6/$S$3</f>
+        <v>13.128134918076242</v>
+      </c>
+      <c r="G6" s="21">
+        <f>lc_detailed!AV6/$S$3</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="21">
+        <f>lc_detailed!AW6/$S$3</f>
+        <v>14.951267446798838</v>
+      </c>
+      <c r="I6" s="21">
+        <f>lc_detailed!AX6/$S$3</f>
+        <v>4.449038910034111</v>
+      </c>
+      <c r="J6" s="21">
+        <f>lc_detailed!AY6/$S$3</f>
+        <v>9.9780772454703719</v>
+      </c>
+      <c r="K6" s="21">
+        <f>lc_detailed!BA6/$S$3</f>
+        <v>-3.8135791923685884</v>
+      </c>
+      <c r="L6" s="21">
+        <f>lc_detailed!BB6/$S$3</f>
+        <v>0</v>
+      </c>
+      <c r="M6" s="21">
+        <f>lc_detailed!AZ6</f>
+        <v>0</v>
+      </c>
+      <c r="N6" s="21">
+        <f>lc_detailed!AN6</f>
+        <v>137.19357300111162</v>
+      </c>
+      <c r="O6" s="21">
+        <f t="shared" si="0"/>
+        <v>38.109325833642117</v>
+      </c>
+      <c r="P6" s="21">
+        <f t="shared" si="1"/>
+        <v>38.109325833642117</v>
+      </c>
+    </row>
+    <row r="7" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B7" s="21" t="str">
+        <f>lc_detailed!AL7</f>
+        <v>SE_Biochemical_CCS_86</v>
+      </c>
+      <c r="C7" s="21" t="str">
+        <f>lc_detailed!AM7</f>
+        <v>Biomass_Agri</v>
+      </c>
+      <c r="D7" s="21">
+        <f>lc_detailed!AS7/$S$3</f>
+        <v>-0.58361349436886112</v>
+      </c>
+      <c r="E7" s="21">
+        <f>lc_detailed!AT7/$S$3</f>
+        <v>1.2366708112135607</v>
+      </c>
+      <c r="F7" s="21">
+        <f>lc_detailed!AU7/$S$3</f>
+        <v>10.691645711092482</v>
+      </c>
+      <c r="G7" s="21">
+        <f>lc_detailed!AV7/$S$3</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="21">
+        <f>lc_detailed!AW7/$S$3</f>
+        <v>16.517339197139297</v>
+      </c>
+      <c r="I7" s="21">
+        <f>lc_detailed!AX7/$S$3</f>
+        <v>5.3058341680868315</v>
+      </c>
+      <c r="J7" s="21">
+        <f>lc_detailed!AY7/$S$3</f>
+        <v>10.191215136730642</v>
+      </c>
+      <c r="K7" s="21">
+        <f>lc_detailed!BA7/$S$3</f>
+        <v>-16.659319629820676</v>
+      </c>
+      <c r="L7" s="21">
+        <f>lc_detailed!BB7/$S$3</f>
+        <v>0</v>
+      </c>
+      <c r="M7" s="21">
+        <f>lc_detailed!AZ7</f>
+        <v>0</v>
+      </c>
+      <c r="N7" s="21">
+        <f>lc_detailed!AN7</f>
+        <v>96.1191788402638</v>
+      </c>
+      <c r="O7" s="21">
+        <f t="shared" si="0"/>
+        <v>26.699771900073276</v>
+      </c>
+      <c r="P7" s="21">
+        <f t="shared" si="1"/>
+        <v>26.699771900073276</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="P2:AB2"/>
-    <mergeCell ref="A2:N2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>